<commit_message>
Cotacoes CEAGESP - coleta de 09/09/2026 17:46
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$393</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$398</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J393"/>
+  <dimension ref="A1:J398"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -17747,8 +17747,228 @@
         </is>
       </c>
     </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F394" s="2" t="n">
+        <v>41.93</v>
+      </c>
+      <c r="G394" s="2" t="n">
+        <v>42.45</v>
+      </c>
+      <c r="H394" s="2" t="n">
+        <v>42.99</v>
+      </c>
+      <c r="I394" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J394" t="inlineStr">
+        <is>
+          <t>09/09/2026 17:46:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F395" s="2" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="G395" s="2" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="H395" s="2" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="I395" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J395" t="inlineStr">
+        <is>
+          <t>09/09/2026 17:46:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F396" s="2" t="n">
+        <v>12.94</v>
+      </c>
+      <c r="G396" s="2" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="H396" s="2" t="n">
+        <v>14.87</v>
+      </c>
+      <c r="I396" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J396" t="inlineStr">
+        <is>
+          <t>09/09/2026 17:46:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F397" s="2" t="n">
+        <v>11.98</v>
+      </c>
+      <c r="G397" s="2" t="n">
+        <v>12.48</v>
+      </c>
+      <c r="H397" s="2" t="n">
+        <v>12.99</v>
+      </c>
+      <c r="I397" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J397" t="inlineStr">
+        <is>
+          <t>09/09/2026 17:46:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F398" s="2" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="G398" s="2" t="n">
+        <v>27.79</v>
+      </c>
+      <c r="H398" s="2" t="n">
+        <v>28.29</v>
+      </c>
+      <c r="I398" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J398" t="inlineStr">
+        <is>
+          <t>09/09/2026 17:46:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J393"/>
+  <autoFilter ref="A1:J398"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17759,7 +17979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -17829,7 +18049,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>04/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -17853,27 +18073,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>40.75</v>
+        <v>41.93</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>41.35</v>
+        <v>42.45</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>41.96</v>
+        <v>42.99</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>04/09/2026 19:55:03</t>
+          <t>09/09/2026 17:46:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>04/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -17910,14 +18130,14 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>04/09/2026 19:55:03</t>
+          <t>09/09/2026 17:46:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>04/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -17941,27 +18161,27 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>12.99</v>
+        <v>12.94</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>13.77</v>
+        <v>13.9</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>14.5</v>
+        <v>14.87</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>04/09/2026 19:55:03</t>
+          <t>09/09/2026 17:46:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>04/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -17985,25 +18205,69 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>11.87</v>
+        <v>11.98</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>12.29</v>
+        <v>12.48</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>12.74</v>
+        <v>12.99</v>
       </c>
       <c r="I5" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>04/09/2026 19:55:03</t>
+          <t>09/09/2026 17:46:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>27.79</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>28.29</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>09/09/2026 17:46:00</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J5"/>
+  <autoFilter ref="A1:J6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 11/09/2026 20:06
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$398</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$404</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J398"/>
+  <dimension ref="A1:J404"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -17967,8 +17967,272 @@
         </is>
       </c>
     </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F399" s="2" t="n">
+        <v>41.01</v>
+      </c>
+      <c r="G399" s="2" t="n">
+        <v>41.66</v>
+      </c>
+      <c r="H399" s="2" t="n">
+        <v>42.3</v>
+      </c>
+      <c r="I399" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J399" t="inlineStr">
+        <is>
+          <t>11/09/2026 20:06:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>PANGASIUS</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F400" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="G400" s="2" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H400" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I400" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J400" t="inlineStr">
+        <is>
+          <t>11/09/2026 20:06:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F401" s="2" t="n">
+        <v>25.67</v>
+      </c>
+      <c r="G401" s="2" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="H401" s="2" t="n">
+        <v>27.33</v>
+      </c>
+      <c r="I401" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J401" t="inlineStr">
+        <is>
+          <t>11/09/2026 20:06:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F402" s="2" t="n">
+        <v>12.28</v>
+      </c>
+      <c r="G402" s="2" t="n">
+        <v>12.93</v>
+      </c>
+      <c r="H402" s="2" t="n">
+        <v>13.57</v>
+      </c>
+      <c r="I402" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J402" t="inlineStr">
+        <is>
+          <t>11/09/2026 20:06:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F403" s="2" t="n">
+        <v>12.18</v>
+      </c>
+      <c r="G403" s="2" t="n">
+        <v>12.49</v>
+      </c>
+      <c r="H403" s="2" t="n">
+        <v>12.93</v>
+      </c>
+      <c r="I403" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J403" t="inlineStr">
+        <is>
+          <t>11/09/2026 20:06:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F404" s="2" t="n">
+        <v>37.6</v>
+      </c>
+      <c r="G404" s="2" t="n">
+        <v>38.4</v>
+      </c>
+      <c r="H404" s="2" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="I404" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J404" t="inlineStr">
+        <is>
+          <t>11/09/2026 20:06:49</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J398"/>
+  <autoFilter ref="A1:J404"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17979,7 +18243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -18049,7 +18313,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -18073,27 +18337,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>41.93</v>
+        <v>41.01</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>42.45</v>
+        <v>41.66</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>42.99</v>
+        <v>42.3</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>09/09/2026 17:46:00</t>
+          <t>11/09/2026 20:06:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -18103,7 +18367,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PINTADO</t>
+          <t>PANGASIUS</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -18117,27 +18381,27 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>26.5</v>
+        <v>9</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>27.5</v>
+        <v>9.5</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>28.5</v>
+        <v>10</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>09/09/2026 17:46:00</t>
+          <t>11/09/2026 20:06:49</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -18147,7 +18411,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>TAMBAQUI</t>
+          <t>PINTADO</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -18161,27 +18425,27 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>12.94</v>
+        <v>25.67</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>13.9</v>
+        <v>26.5</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>14.87</v>
+        <v>27.33</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>09/09/2026 17:46:00</t>
+          <t>11/09/2026 20:06:49</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -18191,7 +18455,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>TILÁPIA</t>
+          <t>TAMBAQUI</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -18205,27 +18469,27 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>11.98</v>
+        <v>12.28</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>12.48</v>
+        <v>12.93</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>12.99</v>
+        <v>13.57</v>
       </c>
       <c r="I5" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>09/09/2026 17:46:00</t>
+          <t>11/09/2026 20:06:49</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -18235,39 +18499,83 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>12.18</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>12.49</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>12.93</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>11/09/2026 20:06:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>TRUTA</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>27.3</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>27.79</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>28.29</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>09/09/2026 17:46:00</t>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>37.6</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>38.4</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>11/09/2026 20:06:49</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J6"/>
+  <autoFilter ref="A1:J7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 14/09/2026 20:46
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$404</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$410</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J404"/>
+  <dimension ref="A1:J410"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -18231,8 +18231,272 @@
         </is>
       </c>
     </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F405" s="2" t="n">
+        <v>40.52</v>
+      </c>
+      <c r="G405" s="2" t="n">
+        <v>41.53</v>
+      </c>
+      <c r="H405" s="2" t="n">
+        <v>42.06</v>
+      </c>
+      <c r="I405" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J405" t="inlineStr">
+        <is>
+          <t>14/09/2026 20:46:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>PANGASIUS</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F406" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G406" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="H406" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I406" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J406" t="inlineStr">
+        <is>
+          <t>14/09/2026 20:46:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F407" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="G407" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="H407" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="I407" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J407" t="inlineStr">
+        <is>
+          <t>14/09/2026 20:46:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F408" s="2" t="n">
+        <v>12.34</v>
+      </c>
+      <c r="G408" s="2" t="n">
+        <v>13.33</v>
+      </c>
+      <c r="H408" s="2" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="I408" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J408" t="inlineStr">
+        <is>
+          <t>14/09/2026 20:46:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F409" s="2" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="G409" s="2" t="n">
+        <v>11.76</v>
+      </c>
+      <c r="H409" s="2" t="n">
+        <v>12.08</v>
+      </c>
+      <c r="I409" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J409" t="inlineStr">
+        <is>
+          <t>14/09/2026 20:46:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F410" s="2" t="n">
+        <v>34.2</v>
+      </c>
+      <c r="G410" s="2" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="H410" s="2" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="I410" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J410" t="inlineStr">
+        <is>
+          <t>14/09/2026 20:46:43</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J404"/>
+  <autoFilter ref="A1:J410"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18313,7 +18577,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -18337,27 +18601,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>41.01</v>
+        <v>40.52</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>41.66</v>
+        <v>41.53</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>42.3</v>
+        <v>42.06</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>11/09/2026 20:06:49</t>
+          <t>14/09/2026 20:46:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -18381,10 +18645,10 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G3" s="2" t="n">
         <v>9</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>9.5</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10</v>
@@ -18394,14 +18658,14 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>11/09/2026 20:06:49</t>
+          <t>14/09/2026 20:46:43</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -18425,27 +18689,27 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>25.67</v>
+        <v>26</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>26.5</v>
+        <v>27</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>27.33</v>
+        <v>28</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>11/09/2026 20:06:49</t>
+          <t>14/09/2026 20:46:43</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -18469,27 +18733,27 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>12.28</v>
+        <v>12.34</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>12.93</v>
+        <v>13.33</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>13.57</v>
+        <v>14.1</v>
       </c>
       <c r="I5" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>11/09/2026 20:06:49</t>
+          <t>14/09/2026 20:46:43</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -18513,27 +18777,27 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>12.18</v>
+        <v>10.75</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>12.49</v>
+        <v>11.76</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>12.93</v>
+        <v>12.08</v>
       </c>
       <c r="I6" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>11/09/2026 20:06:49</t>
+          <t>14/09/2026 20:46:43</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -18557,20 +18821,20 @@
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>37.6</v>
+        <v>34.2</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>38.4</v>
+        <v>35.2</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>39.2</v>
+        <v>36.2</v>
       </c>
       <c r="I7" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>11/09/2026 20:06:49</t>
+          <t>14/09/2026 20:46:43</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 16/09/2026 18:07
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$410</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$413</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J410"/>
+  <dimension ref="A1:J413"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -18495,8 +18495,140 @@
         </is>
       </c>
     </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F411" s="2" t="n">
+        <v>41.35</v>
+      </c>
+      <c r="G411" s="2" t="n">
+        <v>42.13</v>
+      </c>
+      <c r="H411" s="2" t="n">
+        <v>42.89</v>
+      </c>
+      <c r="I411" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J411" t="inlineStr">
+        <is>
+          <t>16/09/2026 18:07:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F412" s="2" t="n">
+        <v>12.28</v>
+      </c>
+      <c r="G412" s="2" t="n">
+        <v>12.43</v>
+      </c>
+      <c r="H412" s="2" t="n">
+        <v>12.57</v>
+      </c>
+      <c r="I412" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J412" t="inlineStr">
+        <is>
+          <t>16/09/2026 18:07:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F413" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="G413" s="2" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="H413" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="I413" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J413" t="inlineStr">
+        <is>
+          <t>16/09/2026 18:07:10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J410"/>
+  <autoFilter ref="A1:J413"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18507,7 +18639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -18577,7 +18709,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>16/09/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -18601,27 +18733,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>40.52</v>
+        <v>41.35</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>41.53</v>
+        <v>42.13</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>42.06</v>
+        <v>42.89</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>14/09/2026 20:46:43</t>
+          <t>16/09/2026 18:07:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>16/09/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -18631,7 +18763,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PANGASIUS</t>
+          <t>TILÁPIA</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -18645,27 +18777,27 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>8</v>
+        <v>12.28</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>9</v>
+        <v>12.43</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>10</v>
+        <v>12.57</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>14/09/2026 20:46:43</t>
+          <t>16/09/2026 18:07:10</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>16/09/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -18675,7 +18807,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PINTADO</t>
+          <t>TRUTA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -18689,157 +18821,25 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>27</v>
+        <v>34.5</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>14/09/2026 20:46:43</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>14/09/2026</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>TAMBAQUI</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>12.34</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>13.33</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>14.1</v>
-      </c>
-      <c r="I5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>14/09/2026 20:46:43</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>14/09/2026</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>TILÁPIA</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>10.75</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>11.76</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>12.08</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>14/09/2026 20:46:43</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>14/09/2026</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>TRUTA</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>34.2</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>35.2</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>36.2</v>
-      </c>
-      <c r="I7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>14/09/2026 20:46:43</t>
+          <t>16/09/2026 18:07:10</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J7"/>
+  <autoFilter ref="A1:J4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 18/09/2026 17:41
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$413</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$418</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J413"/>
+  <dimension ref="A1:J418"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -18627,8 +18627,228 @@
         </is>
       </c>
     </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F414" s="2" t="n">
+        <v>42.7</v>
+      </c>
+      <c r="G414" s="2" t="n">
+        <v>43.6</v>
+      </c>
+      <c r="H414" s="2" t="n">
+        <v>44.51</v>
+      </c>
+      <c r="I414" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J414" t="inlineStr">
+        <is>
+          <t>18/09/2026 17:41:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F415" s="2" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="G415" s="2" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="H415" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I415" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J415" t="inlineStr">
+        <is>
+          <t>18/09/2026 17:41:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F416" s="2" t="n">
+        <v>11.78</v>
+      </c>
+      <c r="G416" s="2" t="n">
+        <v>12.07</v>
+      </c>
+      <c r="H416" s="2" t="n">
+        <v>12.48</v>
+      </c>
+      <c r="I416" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J416" t="inlineStr">
+        <is>
+          <t>18/09/2026 17:41:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F417" s="2" t="n">
+        <v>12.15</v>
+      </c>
+      <c r="G417" s="2" t="n">
+        <v>12.29</v>
+      </c>
+      <c r="H417" s="2" t="n">
+        <v>12.43</v>
+      </c>
+      <c r="I417" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J417" t="inlineStr">
+        <is>
+          <t>18/09/2026 17:41:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F418" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="G418" s="2" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="H418" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="I418" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J418" t="inlineStr">
+        <is>
+          <t>18/09/2026 17:41:53</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J413"/>
+  <autoFilter ref="A1:J418"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18639,7 +18859,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -18709,7 +18929,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>16/09/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -18733,27 +18953,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>41.35</v>
+        <v>42.7</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>42.13</v>
+        <v>43.6</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>42.89</v>
+        <v>44.51</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>16/09/2026 18:07:10</t>
+          <t>18/09/2026 17:41:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>16/09/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -18763,7 +18983,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>TILÁPIA</t>
+          <t>PINTADO</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -18777,27 +18997,27 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>12.28</v>
+        <v>4.8</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>12.43</v>
+        <v>4.9</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>12.57</v>
+        <v>5</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>16/09/2026 18:07:10</t>
+          <t>18/09/2026 17:41:53</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>16/09/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -18807,39 +19027,127 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>11.78</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>12.07</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>12.48</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>18/09/2026 17:41:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>12.15</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>12.29</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>12.43</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>18/09/2026 17:41:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>TRUTA</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>34</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>34.5</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="I4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>16/09/2026 18:07:10</t>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>18/09/2026 17:41:53</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J4"/>
+  <autoFilter ref="A1:J6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 21/09/2026 20:58
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$418</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$420</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J418"/>
+  <dimension ref="A1:J420"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -18847,8 +18847,96 @@
         </is>
       </c>
     </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>21/09/2026</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F419" s="2" t="n">
+        <v>40.7</v>
+      </c>
+      <c r="G419" s="2" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="H419" s="2" t="n">
+        <v>41.89</v>
+      </c>
+      <c r="I419" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J419" t="inlineStr">
+        <is>
+          <t>21/09/2026 20:58:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>21/09/2026</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F420" s="2" t="n">
+        <v>11.83</v>
+      </c>
+      <c r="G420" s="2" t="n">
+        <v>12.22</v>
+      </c>
+      <c r="H420" s="2" t="n">
+        <v>12.67</v>
+      </c>
+      <c r="I420" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J420" t="inlineStr">
+        <is>
+          <t>21/09/2026 20:58:13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J418"/>
+  <autoFilter ref="A1:J420"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18859,7 +18947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -18929,7 +19017,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>21/09/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -18953,27 +19041,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>42.7</v>
+        <v>40.7</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>43.6</v>
+        <v>41.3</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>44.51</v>
+        <v>41.89</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>18/09/2026 17:41:53</t>
+          <t>21/09/2026 20:58:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>21/09/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -18983,7 +19071,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PINTADO</t>
+          <t>TILÁPIA</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -18997,157 +19085,25 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>4.8</v>
+        <v>11.83</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.9</v>
+        <v>12.22</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>5</v>
+        <v>12.67</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>18/09/2026 17:41:53</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>18/09/2026</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>TAMBAQUI</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>11.78</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>12.07</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>12.48</v>
-      </c>
-      <c r="I4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>18/09/2026 17:41:53</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>18/09/2026</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>TILÁPIA</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>12.15</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>12.29</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>12.43</v>
-      </c>
-      <c r="I5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>18/09/2026 17:41:53</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>18/09/2026</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>TRUTA</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>37</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>18/09/2026 17:41:53</t>
+          <t>21/09/2026 20:58:13</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J6"/>
+  <autoFilter ref="A1:J3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 23/09/2026 18:20
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$420</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$422</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J420"/>
+  <dimension ref="A1:J422"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -18935,8 +18935,96 @@
         </is>
       </c>
     </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>23/09/2026</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F421" s="2" t="n">
+        <v>41.95</v>
+      </c>
+      <c r="G421" s="2" t="n">
+        <v>42.48</v>
+      </c>
+      <c r="H421" s="2" t="n">
+        <v>43.04</v>
+      </c>
+      <c r="I421" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J421" t="inlineStr">
+        <is>
+          <t>23/09/2026 18:20:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>23/09/2026</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F422" s="2" t="n">
+        <v>12.02</v>
+      </c>
+      <c r="G422" s="2" t="n">
+        <v>12.32</v>
+      </c>
+      <c r="H422" s="2" t="n">
+        <v>12.54</v>
+      </c>
+      <c r="I422" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J422" t="inlineStr">
+        <is>
+          <t>23/09/2026 18:20:17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J420"/>
+  <autoFilter ref="A1:J422"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19017,7 +19105,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>21/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -19041,27 +19129,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>40.7</v>
+        <v>41.95</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>41.3</v>
+        <v>42.48</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>41.89</v>
+        <v>43.04</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>21/09/2026 20:58:13</t>
+          <t>23/09/2026 18:20:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>21/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -19085,20 +19173,20 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>11.83</v>
+        <v>12.02</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>12.22</v>
+        <v>12.32</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>12.67</v>
+        <v>12.54</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>21/09/2026 20:58:13</t>
+          <t>23/09/2026 18:20:17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 28/09/2026 10:26
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$422</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$427</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J422"/>
+  <dimension ref="A1:J427"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -19023,8 +19023,228 @@
         </is>
       </c>
     </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F423" s="2" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="G423" s="2" t="n">
+        <v>43.05</v>
+      </c>
+      <c r="H423" s="2" t="n">
+        <v>43.73</v>
+      </c>
+      <c r="I423" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J423" t="inlineStr">
+        <is>
+          <t>28/09/2026 10:26:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F424" s="2" t="n">
+        <v>23.08</v>
+      </c>
+      <c r="G424" s="2" t="n">
+        <v>23.58</v>
+      </c>
+      <c r="H424" s="2" t="n">
+        <v>24.07</v>
+      </c>
+      <c r="I424" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J424" t="inlineStr">
+        <is>
+          <t>28/09/2026 10:26:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F425" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="G425" s="2" t="n">
+        <v>13.83</v>
+      </c>
+      <c r="H425" s="2" t="n">
+        <v>14.67</v>
+      </c>
+      <c r="I425" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J425" t="inlineStr">
+        <is>
+          <t>28/09/2026 10:26:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F426" s="2" t="n">
+        <v>12.19</v>
+      </c>
+      <c r="G426" s="2" t="n">
+        <v>12.32</v>
+      </c>
+      <c r="H426" s="2" t="n">
+        <v>12.44</v>
+      </c>
+      <c r="I426" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J426" t="inlineStr">
+        <is>
+          <t>28/09/2026 10:26:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F427" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="G427" s="2" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="H427" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="I427" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J427" t="inlineStr">
+        <is>
+          <t>28/09/2026 10:26:45</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J422"/>
+  <autoFilter ref="A1:J427"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19035,7 +19255,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -19105,7 +19325,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
+          <t>25/09/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -19129,27 +19349,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>41.95</v>
+        <v>42.2</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>42.48</v>
+        <v>43.05</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>43.04</v>
+        <v>43.73</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>23/09/2026 18:20:17</t>
+          <t>28/09/2026 10:26:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
+          <t>25/09/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -19159,39 +19379,171 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>23.08</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>23.58</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>24.07</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>28/09/2026 10:26:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>13.83</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>14.67</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>28/09/2026 10:26:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>TILÁPIA</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>12.02</v>
-      </c>
-      <c r="G3" s="2" t="n">
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>12.19</v>
+      </c>
+      <c r="G5" s="2" t="n">
         <v>12.32</v>
       </c>
-      <c r="H3" s="2" t="n">
-        <v>12.54</v>
-      </c>
-      <c r="I3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>23/09/2026 18:20:17</t>
+      <c r="H5" s="2" t="n">
+        <v>12.44</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>28/09/2026 10:26:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>28/09/2026 10:26:45</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J3"/>
+  <autoFilter ref="A1:J6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 29/09/2026 02:11
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$427</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$432</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J427"/>
+  <dimension ref="A1:J432"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -19243,8 +19243,228 @@
         </is>
       </c>
     </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F428" s="2" t="n">
+        <v>36.93</v>
+      </c>
+      <c r="G428" s="2" t="n">
+        <v>39.52</v>
+      </c>
+      <c r="H428" s="2" t="n">
+        <v>41.48</v>
+      </c>
+      <c r="I428" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J428" t="inlineStr">
+        <is>
+          <t>29/09/2026 02:11:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F429" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="G429" s="2" t="n">
+        <v>22.07</v>
+      </c>
+      <c r="H429" s="2" t="n">
+        <v>24.07</v>
+      </c>
+      <c r="I429" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J429" t="inlineStr">
+        <is>
+          <t>29/09/2026 02:11:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F430" s="2" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="G430" s="2" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="H430" s="2" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="I430" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J430" t="inlineStr">
+        <is>
+          <t>29/09/2026 02:11:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F431" s="2" t="n">
+        <v>10.93</v>
+      </c>
+      <c r="G431" s="2" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="H431" s="2" t="n">
+        <v>12.61</v>
+      </c>
+      <c r="I431" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J431" t="inlineStr">
+        <is>
+          <t>29/09/2026 02:11:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F432" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="G432" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="H432" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I432" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J432" t="inlineStr">
+        <is>
+          <t>29/09/2026 02:11:46</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J427"/>
+  <autoFilter ref="A1:J432"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19325,7 +19545,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>25/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -19349,27 +19569,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>42.2</v>
+        <v>36.93</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>43.05</v>
+        <v>39.52</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>43.73</v>
+        <v>41.48</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>28/09/2026 10:26:45</t>
+          <t>29/09/2026 02:11:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>25/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -19393,10 +19613,10 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>23.08</v>
+        <v>20</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>23.58</v>
+        <v>22.07</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>24.07</v>
@@ -19406,14 +19626,14 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>28/09/2026 10:26:45</t>
+          <t>29/09/2026 02:11:46</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>25/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -19437,27 +19657,27 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>13</v>
+        <v>13.5</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>13.83</v>
+        <v>14.5</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>14.67</v>
+        <v>15.5</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>28/09/2026 10:26:45</t>
+          <t>29/09/2026 02:11:46</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>25/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -19481,27 +19701,27 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>12.19</v>
+        <v>10.93</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>12.32</v>
+        <v>11.9</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>12.44</v>
+        <v>12.61</v>
       </c>
       <c r="I5" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>28/09/2026 10:26:45</t>
+          <t>29/09/2026 02:11:46</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>25/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -19525,20 +19745,20 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>34.5</v>
+        <v>29</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="I6" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>28/09/2026 10:26:45</t>
+          <t>29/09/2026 02:11:46</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 30/09/2026 15:21
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$432</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$431</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J432"/>
+  <dimension ref="A1:J431"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -18667,7 +18667,7 @@
       </c>
       <c r="J414" t="inlineStr">
         <is>
-          <t>18/09/2026 17:41:53</t>
+          <t>30/09/2026 15:21:34</t>
         </is>
       </c>
     </row>
@@ -18684,7 +18684,7 @@
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>PINTADO</t>
+          <t>TAMBAQUI</t>
         </is>
       </c>
       <c r="D415" t="inlineStr">
@@ -18698,20 +18698,20 @@
         </is>
       </c>
       <c r="F415" s="2" t="n">
-        <v>4.8</v>
+        <v>11.78</v>
       </c>
       <c r="G415" s="2" t="n">
-        <v>4.9</v>
+        <v>12.07</v>
       </c>
       <c r="H415" s="2" t="n">
-        <v>5</v>
+        <v>12.48</v>
       </c>
       <c r="I415" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J415" t="inlineStr">
         <is>
-          <t>18/09/2026 17:41:53</t>
+          <t>30/09/2026 15:21:34</t>
         </is>
       </c>
     </row>
@@ -18728,7 +18728,7 @@
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>TAMBAQUI</t>
+          <t>TILÁPIA</t>
         </is>
       </c>
       <c r="D416" t="inlineStr">
@@ -18742,20 +18742,20 @@
         </is>
       </c>
       <c r="F416" s="2" t="n">
-        <v>11.78</v>
+        <v>12.15</v>
       </c>
       <c r="G416" s="2" t="n">
-        <v>12.07</v>
+        <v>12.29</v>
       </c>
       <c r="H416" s="2" t="n">
-        <v>12.48</v>
+        <v>12.43</v>
       </c>
       <c r="I416" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J416" t="inlineStr">
         <is>
-          <t>18/09/2026 17:41:53</t>
+          <t>30/09/2026 15:21:34</t>
         </is>
       </c>
     </row>
@@ -18772,7 +18772,7 @@
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>TILÁPIA</t>
+          <t>TRUTA</t>
         </is>
       </c>
       <c r="D417" t="inlineStr">
@@ -18786,27 +18786,27 @@
         </is>
       </c>
       <c r="F417" s="2" t="n">
-        <v>12.15</v>
+        <v>37</v>
       </c>
       <c r="G417" s="2" t="n">
-        <v>12.29</v>
+        <v>37.5</v>
       </c>
       <c r="H417" s="2" t="n">
-        <v>12.43</v>
+        <v>38</v>
       </c>
       <c r="I417" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J417" t="inlineStr">
         <is>
-          <t>18/09/2026 17:41:53</t>
+          <t>30/09/2026 15:21:34</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>21/09/2026</t>
         </is>
       </c>
       <c r="B418" t="inlineStr">
@@ -18816,7 +18816,7 @@
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>TRUTA</t>
+          <t>FILE DE TILAPIA</t>
         </is>
       </c>
       <c r="D418" t="inlineStr">
@@ -18830,20 +18830,20 @@
         </is>
       </c>
       <c r="F418" s="2" t="n">
-        <v>37</v>
+        <v>40.7</v>
       </c>
       <c r="G418" s="2" t="n">
-        <v>37.5</v>
+        <v>41.3</v>
       </c>
       <c r="H418" s="2" t="n">
-        <v>38</v>
+        <v>41.89</v>
       </c>
       <c r="I418" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J418" t="inlineStr">
         <is>
-          <t>18/09/2026 17:41:53</t>
+          <t>21/09/2026 20:58:13</t>
         </is>
       </c>
     </row>
@@ -18860,7 +18860,7 @@
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>FILE DE TILAPIA</t>
+          <t>TILÁPIA</t>
         </is>
       </c>
       <c r="D419" t="inlineStr">
@@ -18874,13 +18874,13 @@
         </is>
       </c>
       <c r="F419" s="2" t="n">
-        <v>40.7</v>
+        <v>11.83</v>
       </c>
       <c r="G419" s="2" t="n">
-        <v>41.3</v>
+        <v>12.22</v>
       </c>
       <c r="H419" s="2" t="n">
-        <v>41.89</v>
+        <v>12.67</v>
       </c>
       <c r="I419" s="2" t="n">
         <v>1</v>
@@ -18894,7 +18894,7 @@
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>21/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="B420" t="inlineStr">
@@ -18904,7 +18904,7 @@
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>TILÁPIA</t>
+          <t>FILE DE TILAPIA</t>
         </is>
       </c>
       <c r="D420" t="inlineStr">
@@ -18918,20 +18918,20 @@
         </is>
       </c>
       <c r="F420" s="2" t="n">
-        <v>11.83</v>
+        <v>41.95</v>
       </c>
       <c r="G420" s="2" t="n">
-        <v>12.22</v>
+        <v>42.48</v>
       </c>
       <c r="H420" s="2" t="n">
-        <v>12.67</v>
+        <v>43.04</v>
       </c>
       <c r="I420" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J420" t="inlineStr">
         <is>
-          <t>21/09/2026 20:58:13</t>
+          <t>23/09/2026 18:20:17</t>
         </is>
       </c>
     </row>
@@ -18948,7 +18948,7 @@
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>FILE DE TILAPIA</t>
+          <t>TILÁPIA</t>
         </is>
       </c>
       <c r="D421" t="inlineStr">
@@ -18962,13 +18962,13 @@
         </is>
       </c>
       <c r="F421" s="2" t="n">
-        <v>41.95</v>
+        <v>12.02</v>
       </c>
       <c r="G421" s="2" t="n">
-        <v>42.48</v>
+        <v>12.32</v>
       </c>
       <c r="H421" s="2" t="n">
-        <v>43.04</v>
+        <v>12.54</v>
       </c>
       <c r="I421" s="2" t="n">
         <v>1</v>
@@ -18982,7 +18982,7 @@
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
+          <t>25/09/2026</t>
         </is>
       </c>
       <c r="B422" t="inlineStr">
@@ -18992,7 +18992,7 @@
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>TILÁPIA</t>
+          <t>FILE DE TILAPIA</t>
         </is>
       </c>
       <c r="D422" t="inlineStr">
@@ -19006,20 +19006,20 @@
         </is>
       </c>
       <c r="F422" s="2" t="n">
-        <v>12.02</v>
+        <v>42.2</v>
       </c>
       <c r="G422" s="2" t="n">
-        <v>12.32</v>
+        <v>43.05</v>
       </c>
       <c r="H422" s="2" t="n">
-        <v>12.54</v>
+        <v>43.73</v>
       </c>
       <c r="I422" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J422" t="inlineStr">
         <is>
-          <t>23/09/2026 18:20:17</t>
+          <t>28/09/2026 10:26:45</t>
         </is>
       </c>
     </row>
@@ -19036,7 +19036,7 @@
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>FILE DE TILAPIA</t>
+          <t>PINTADO</t>
         </is>
       </c>
       <c r="D423" t="inlineStr">
@@ -19050,13 +19050,13 @@
         </is>
       </c>
       <c r="F423" s="2" t="n">
-        <v>42.2</v>
+        <v>23.08</v>
       </c>
       <c r="G423" s="2" t="n">
-        <v>43.05</v>
+        <v>23.58</v>
       </c>
       <c r="H423" s="2" t="n">
-        <v>43.73</v>
+        <v>24.07</v>
       </c>
       <c r="I423" s="2" t="n">
         <v>1</v>
@@ -19080,7 +19080,7 @@
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>PINTADO</t>
+          <t>TAMBAQUI</t>
         </is>
       </c>
       <c r="D424" t="inlineStr">
@@ -19094,13 +19094,13 @@
         </is>
       </c>
       <c r="F424" s="2" t="n">
-        <v>23.08</v>
+        <v>13</v>
       </c>
       <c r="G424" s="2" t="n">
-        <v>23.58</v>
+        <v>13.83</v>
       </c>
       <c r="H424" s="2" t="n">
-        <v>24.07</v>
+        <v>14.67</v>
       </c>
       <c r="I424" s="2" t="n">
         <v>1</v>
@@ -19124,7 +19124,7 @@
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>TAMBAQUI</t>
+          <t>TILÁPIA</t>
         </is>
       </c>
       <c r="D425" t="inlineStr">
@@ -19138,13 +19138,13 @@
         </is>
       </c>
       <c r="F425" s="2" t="n">
-        <v>13</v>
+        <v>12.19</v>
       </c>
       <c r="G425" s="2" t="n">
-        <v>13.83</v>
+        <v>12.32</v>
       </c>
       <c r="H425" s="2" t="n">
-        <v>14.67</v>
+        <v>12.44</v>
       </c>
       <c r="I425" s="2" t="n">
         <v>1</v>
@@ -19168,7 +19168,7 @@
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>TILÁPIA</t>
+          <t>TRUTA</t>
         </is>
       </c>
       <c r="D426" t="inlineStr">
@@ -19182,13 +19182,13 @@
         </is>
       </c>
       <c r="F426" s="2" t="n">
-        <v>12.19</v>
+        <v>34</v>
       </c>
       <c r="G426" s="2" t="n">
-        <v>12.32</v>
+        <v>34.5</v>
       </c>
       <c r="H426" s="2" t="n">
-        <v>12.44</v>
+        <v>35</v>
       </c>
       <c r="I426" s="2" t="n">
         <v>1</v>
@@ -19202,7 +19202,7 @@
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>25/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="B427" t="inlineStr">
@@ -19212,7 +19212,7 @@
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>TRUTA</t>
+          <t>FILE DE TILAPIA</t>
         </is>
       </c>
       <c r="D427" t="inlineStr">
@@ -19226,20 +19226,20 @@
         </is>
       </c>
       <c r="F427" s="2" t="n">
-        <v>34</v>
+        <v>36.93</v>
       </c>
       <c r="G427" s="2" t="n">
-        <v>34.5</v>
+        <v>39.52</v>
       </c>
       <c r="H427" s="2" t="n">
-        <v>35</v>
+        <v>41.48</v>
       </c>
       <c r="I427" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J427" t="inlineStr">
         <is>
-          <t>28/09/2026 10:26:45</t>
+          <t>29/09/2026 02:11:46</t>
         </is>
       </c>
     </row>
@@ -19256,7 +19256,7 @@
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>FILE DE TILAPIA</t>
+          <t>PINTADO</t>
         </is>
       </c>
       <c r="D428" t="inlineStr">
@@ -19270,13 +19270,13 @@
         </is>
       </c>
       <c r="F428" s="2" t="n">
-        <v>36.93</v>
+        <v>20</v>
       </c>
       <c r="G428" s="2" t="n">
-        <v>39.52</v>
+        <v>22.07</v>
       </c>
       <c r="H428" s="2" t="n">
-        <v>41.48</v>
+        <v>24.07</v>
       </c>
       <c r="I428" s="2" t="n">
         <v>1</v>
@@ -19300,7 +19300,7 @@
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>PINTADO</t>
+          <t>TAMBAQUI</t>
         </is>
       </c>
       <c r="D429" t="inlineStr">
@@ -19314,13 +19314,13 @@
         </is>
       </c>
       <c r="F429" s="2" t="n">
-        <v>20</v>
+        <v>13.5</v>
       </c>
       <c r="G429" s="2" t="n">
-        <v>22.07</v>
+        <v>14.5</v>
       </c>
       <c r="H429" s="2" t="n">
-        <v>24.07</v>
+        <v>15.5</v>
       </c>
       <c r="I429" s="2" t="n">
         <v>1</v>
@@ -19344,7 +19344,7 @@
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>TAMBAQUI</t>
+          <t>TILÁPIA</t>
         </is>
       </c>
       <c r="D430" t="inlineStr">
@@ -19358,13 +19358,13 @@
         </is>
       </c>
       <c r="F430" s="2" t="n">
-        <v>13.5</v>
+        <v>10.93</v>
       </c>
       <c r="G430" s="2" t="n">
-        <v>14.5</v>
+        <v>11.9</v>
       </c>
       <c r="H430" s="2" t="n">
-        <v>15.5</v>
+        <v>12.61</v>
       </c>
       <c r="I430" s="2" t="n">
         <v>1</v>
@@ -19388,7 +19388,7 @@
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>TILÁPIA</t>
+          <t>TRUTA</t>
         </is>
       </c>
       <c r="D431" t="inlineStr">
@@ -19402,13 +19402,13 @@
         </is>
       </c>
       <c r="F431" s="2" t="n">
-        <v>10.93</v>
+        <v>28</v>
       </c>
       <c r="G431" s="2" t="n">
-        <v>11.9</v>
+        <v>29</v>
       </c>
       <c r="H431" s="2" t="n">
-        <v>12.61</v>
+        <v>30</v>
       </c>
       <c r="I431" s="2" t="n">
         <v>1</v>
@@ -19419,52 +19419,8 @@
         </is>
       </c>
     </row>
-    <row r="432">
-      <c r="A432" t="inlineStr">
-        <is>
-          <t>28/09/2026</t>
-        </is>
-      </c>
-      <c r="B432" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C432" t="inlineStr">
-        <is>
-          <t>TRUTA</t>
-        </is>
-      </c>
-      <c r="D432" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E432" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F432" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="G432" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="H432" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I432" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J432" t="inlineStr">
-        <is>
-          <t>29/09/2026 02:11:46</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J432"/>
+  <autoFilter ref="A1:J431"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 30/09/2026 19:04
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$431</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$435</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J431"/>
+  <dimension ref="A1:J435"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -19419,8 +19419,184 @@
         </is>
       </c>
     </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F432" s="2" t="n">
+        <v>40.29</v>
+      </c>
+      <c r="G432" s="2" t="n">
+        <v>40.88</v>
+      </c>
+      <c r="H432" s="2" t="n">
+        <v>41.48</v>
+      </c>
+      <c r="I432" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J432" t="inlineStr">
+        <is>
+          <t>30/09/2026 19:04:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F433" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G433" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="H433" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="I433" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J433" t="inlineStr">
+        <is>
+          <t>30/09/2026 19:04:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F434" s="2" t="n">
+        <v>12.19</v>
+      </c>
+      <c r="G434" s="2" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="H434" s="2" t="n">
+        <v>12.68</v>
+      </c>
+      <c r="I434" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J434" t="inlineStr">
+        <is>
+          <t>30/09/2026 19:04:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F435" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="G435" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="H435" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="I435" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J435" t="inlineStr">
+        <is>
+          <t>30/09/2026 19:04:47</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J431"/>
+  <autoFilter ref="A1:J435"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19431,7 +19607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -19501,7 +19677,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -19525,10 +19701,10 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>36.93</v>
+        <v>40.29</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>39.52</v>
+        <v>40.88</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>41.48</v>
@@ -19538,14 +19714,14 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>29/09/2026 02:11:46</t>
+          <t>30/09/2026 19:04:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -19555,7 +19731,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PINTADO</t>
+          <t>TAMBAQUI</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -19569,27 +19745,27 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>22.07</v>
+        <v>11</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>24.07</v>
+        <v>12</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>29/09/2026 02:11:46</t>
+          <t>30/09/2026 19:04:47</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -19599,7 +19775,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>TAMBAQUI</t>
+          <t>TILÁPIA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -19613,27 +19789,27 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>13.5</v>
+        <v>12.19</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>14.5</v>
+        <v>12.45</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>15.5</v>
+        <v>12.68</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>29/09/2026 02:11:46</t>
+          <t>30/09/2026 19:04:47</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -19643,7 +19819,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>TILÁPIA</t>
+          <t>TRUTA</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -19657,69 +19833,25 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>10.93</v>
+        <v>38</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>11.9</v>
+        <v>39</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>12.61</v>
+        <v>40</v>
       </c>
       <c r="I5" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>29/09/2026 02:11:46</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>28/09/2026</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>TRUTA</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>29/09/2026 02:11:46</t>
+          <t>30/09/2026 19:04:47</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J6"/>
+  <autoFilter ref="A1:J5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 02/10/2026 19:01
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$435</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$440</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J435"/>
+  <dimension ref="A1:J440"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -19595,8 +19595,228 @@
         </is>
       </c>
     </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F436" s="2" t="n">
+        <v>41.23</v>
+      </c>
+      <c r="G436" s="2" t="n">
+        <v>41.96</v>
+      </c>
+      <c r="H436" s="2" t="n">
+        <v>42.7</v>
+      </c>
+      <c r="I436" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J436" t="inlineStr">
+        <is>
+          <t>02/10/2026 19:01:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F437" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="G437" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="H437" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="I437" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J437" t="inlineStr">
+        <is>
+          <t>02/10/2026 19:01:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F438" s="2" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="G438" s="2" t="n">
+        <v>13.25</v>
+      </c>
+      <c r="H438" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="I438" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J438" t="inlineStr">
+        <is>
+          <t>02/10/2026 19:01:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F439" s="2" t="n">
+        <v>11.89</v>
+      </c>
+      <c r="G439" s="2" t="n">
+        <v>12.18</v>
+      </c>
+      <c r="H439" s="2" t="n">
+        <v>12.42</v>
+      </c>
+      <c r="I439" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J439" t="inlineStr">
+        <is>
+          <t>02/10/2026 19:01:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F440" s="2" t="n">
+        <v>36.59</v>
+      </c>
+      <c r="G440" s="2" t="n">
+        <v>37.59</v>
+      </c>
+      <c r="H440" s="2" t="n">
+        <v>38.58</v>
+      </c>
+      <c r="I440" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J440" t="inlineStr">
+        <is>
+          <t>02/10/2026 19:01:46</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J435"/>
+  <autoFilter ref="A1:J440"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19607,7 +19827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -19677,7 +19897,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>02/10/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -19701,27 +19921,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>40.29</v>
+        <v>41.23</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>40.88</v>
+        <v>41.96</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>41.48</v>
+        <v>42.7</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>30/09/2026 19:04:47</t>
+          <t>02/10/2026 19:01:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>02/10/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -19731,7 +19951,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>TAMBAQUI</t>
+          <t>PINTADO</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -19745,27 +19965,27 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>30/09/2026 19:04:47</t>
+          <t>02/10/2026 19:01:46</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>02/10/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -19775,7 +19995,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>TILÁPIA</t>
+          <t>TAMBAQUI</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -19789,27 +20009,27 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>12.19</v>
+        <v>12.5</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>12.45</v>
+        <v>13.25</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>12.68</v>
+        <v>14</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>30/09/2026 19:04:47</t>
+          <t>02/10/2026 19:01:46</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>02/10/2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -19819,39 +20039,83 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>11.89</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>12.18</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>12.42</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>02/10/2026 19:01:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>TRUTA</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="I5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>30/09/2026 19:04:47</t>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>36.59</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>37.59</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>38.58</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>02/10/2026 19:01:46</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J5"/>
+  <autoFilter ref="A1:J6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 05/10/2026 18:55
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$440</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$445</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J440"/>
+  <dimension ref="A1:J445"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -19815,8 +19815,228 @@
         </is>
       </c>
     </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F441" s="2" t="n">
+        <v>40.91</v>
+      </c>
+      <c r="G441" s="2" t="n">
+        <v>41.55</v>
+      </c>
+      <c r="H441" s="2" t="n">
+        <v>42.21</v>
+      </c>
+      <c r="I441" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J441" t="inlineStr">
+        <is>
+          <t>05/10/2026 18:55:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F442" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="G442" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="H442" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="I442" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J442" t="inlineStr">
+        <is>
+          <t>05/10/2026 18:55:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F443" s="2" t="n">
+        <v>11.75</v>
+      </c>
+      <c r="G443" s="2" t="n">
+        <v>12.35</v>
+      </c>
+      <c r="H443" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="I443" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J443" t="inlineStr">
+        <is>
+          <t>05/10/2026 18:55:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F444" s="2" t="n">
+        <v>11.86</v>
+      </c>
+      <c r="G444" s="2" t="n">
+        <v>12.15</v>
+      </c>
+      <c r="H444" s="2" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="I444" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J444" t="inlineStr">
+        <is>
+          <t>05/10/2026 18:55:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F445" s="2" t="n">
+        <v>36.59</v>
+      </c>
+      <c r="G445" s="2" t="n">
+        <v>37.59</v>
+      </c>
+      <c r="H445" s="2" t="n">
+        <v>38.58</v>
+      </c>
+      <c r="I445" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J445" t="inlineStr">
+        <is>
+          <t>05/10/2026 18:55:20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J440"/>
+  <autoFilter ref="A1:J445"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19897,7 +20117,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>02/10/2026</t>
+          <t>05/10/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -19921,27 +20141,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>41.23</v>
+        <v>40.91</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>41.96</v>
+        <v>41.55</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>42.7</v>
+        <v>42.21</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>02/10/2026 19:01:46</t>
+          <t>05/10/2026 18:55:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>02/10/2026</t>
+          <t>05/10/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -19978,14 +20198,14 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>02/10/2026 19:01:46</t>
+          <t>05/10/2026 18:55:20</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>02/10/2026</t>
+          <t>05/10/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -20009,27 +20229,27 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>12.5</v>
+        <v>11.75</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>13.25</v>
+        <v>12.35</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>02/10/2026 19:01:46</t>
+          <t>05/10/2026 18:55:20</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>02/10/2026</t>
+          <t>05/10/2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -20053,27 +20273,27 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>11.89</v>
+        <v>11.86</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>12.18</v>
+        <v>12.15</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>12.42</v>
+        <v>12.4</v>
       </c>
       <c r="I5" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>02/10/2026 19:01:46</t>
+          <t>05/10/2026 18:55:20</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02/10/2026</t>
+          <t>05/10/2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -20110,7 +20330,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>02/10/2026 19:01:46</t>
+          <t>05/10/2026 18:55:20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 07/10/2026 21:52
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$445</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$448</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J445"/>
+  <dimension ref="A1:J448"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -20035,8 +20035,140 @@
         </is>
       </c>
     </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F446" s="2" t="n">
+        <v>43.55</v>
+      </c>
+      <c r="G446" s="2" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="H446" s="2" t="n">
+        <v>45.44</v>
+      </c>
+      <c r="I446" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J446" t="inlineStr">
+        <is>
+          <t>07/10/2026 21:52:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F447" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="G447" s="2" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H447" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="I447" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J447" t="inlineStr">
+        <is>
+          <t>07/10/2026 21:52:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F448" s="2" t="n">
+        <v>10.65</v>
+      </c>
+      <c r="G448" s="2" t="n">
+        <v>11.04</v>
+      </c>
+      <c r="H448" s="2" t="n">
+        <v>11.38</v>
+      </c>
+      <c r="I448" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J448" t="inlineStr">
+        <is>
+          <t>07/10/2026 21:52:13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J445"/>
+  <autoFilter ref="A1:J448"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -20047,7 +20179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -20117,7 +20249,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>05/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -20141,27 +20273,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>40.91</v>
+        <v>43.55</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>41.55</v>
+        <v>44.5</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>42.21</v>
+        <v>45.44</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>05/10/2026 18:55:20</t>
+          <t>07/10/2026 21:52:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>05/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -20171,7 +20303,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PINTADO</t>
+          <t>TAMBAQUI</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -20185,27 +20317,27 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>27</v>
+        <v>11.5</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>05/10/2026 18:55:20</t>
+          <t>07/10/2026 21:52:13</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>05/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -20215,7 +20347,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>TAMBAQUI</t>
+          <t>TILÁPIA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -20229,113 +20361,25 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>11.75</v>
+        <v>10.65</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>12.35</v>
+        <v>11.04</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>13</v>
+        <v>11.38</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>05/10/2026 18:55:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>05/10/2026</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>TILÁPIA</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>11.86</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>12.15</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>12.4</v>
-      </c>
-      <c r="I5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>05/10/2026 18:55:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>05/10/2026</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>TRUTA</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>36.59</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>37.59</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>38.58</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>05/10/2026 18:55:20</t>
+          <t>07/10/2026 21:52:13</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J6"/>
+  <autoFilter ref="A1:J4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 09/10/2026 21:38
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$448</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$453</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J448"/>
+  <dimension ref="A1:J453"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -20167,8 +20167,228 @@
         </is>
       </c>
     </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F449" s="2" t="n">
+        <v>42.67</v>
+      </c>
+      <c r="G449" s="2" t="n">
+        <v>43.61</v>
+      </c>
+      <c r="H449" s="2" t="n">
+        <v>44.53</v>
+      </c>
+      <c r="I449" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J449" t="inlineStr">
+        <is>
+          <t>09/10/2026 21:38:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>PANGASIUS</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F450" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="G450" s="2" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H450" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I450" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J450" t="inlineStr">
+        <is>
+          <t>09/10/2026 21:38:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F451" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="G451" s="2" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H451" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="I451" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J451" t="inlineStr">
+        <is>
+          <t>09/10/2026 21:38:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F452" s="2" t="n">
+        <v>11.71</v>
+      </c>
+      <c r="G452" s="2" t="n">
+        <v>12.08</v>
+      </c>
+      <c r="H452" s="2" t="n">
+        <v>12.39</v>
+      </c>
+      <c r="I452" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J452" t="inlineStr">
+        <is>
+          <t>09/10/2026 21:38:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F453" s="2" t="n">
+        <v>34.2</v>
+      </c>
+      <c r="G453" s="2" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="H453" s="2" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="I453" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J453" t="inlineStr">
+        <is>
+          <t>09/10/2026 21:38:41</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J448"/>
+  <autoFilter ref="A1:J453"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -20179,7 +20399,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -20249,7 +20469,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -20273,27 +20493,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>43.55</v>
+        <v>42.67</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>44.5</v>
+        <v>43.61</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>45.44</v>
+        <v>44.53</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>07/10/2026 21:52:13</t>
+          <t>09/10/2026 21:38:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -20303,7 +20523,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>TAMBAQUI</t>
+          <t>PANGASIUS</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -20317,27 +20537,27 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>11.5</v>
+        <v>9.5</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>07/10/2026 21:52:13</t>
+          <t>09/10/2026 21:38:41</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -20347,39 +20567,127 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>09/10/2026 21:38:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>TILÁPIA</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>10.65</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>11.04</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>11.38</v>
-      </c>
-      <c r="I4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>07/10/2026 21:52:13</t>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>11.71</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>12.08</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>12.39</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>09/10/2026 21:38:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>34.2</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>09/10/2026 21:38:41</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J4"/>
+  <autoFilter ref="A1:J6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 14/10/2026 18:28
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$453</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$456</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J453"/>
+  <dimension ref="A1:J456"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -20387,8 +20387,140 @@
         </is>
       </c>
     </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>14/10/2026</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F454" s="2" t="n">
+        <v>41.9</v>
+      </c>
+      <c r="G454" s="2" t="n">
+        <v>42.42</v>
+      </c>
+      <c r="H454" s="2" t="n">
+        <v>42.91</v>
+      </c>
+      <c r="I454" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J454" t="inlineStr">
+        <is>
+          <t>14/10/2026 18:28:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>14/10/2026</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F455" s="2" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="G455" s="2" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="H455" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="I455" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J455" t="inlineStr">
+        <is>
+          <t>14/10/2026 18:28:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>14/10/2026</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F456" s="2" t="n">
+        <v>11.87</v>
+      </c>
+      <c r="G456" s="2" t="n">
+        <v>12.14</v>
+      </c>
+      <c r="H456" s="2" t="n">
+        <v>12.38</v>
+      </c>
+      <c r="I456" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J456" t="inlineStr">
+        <is>
+          <t>14/10/2026 18:28:17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J453"/>
+  <autoFilter ref="A1:J456"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -20399,7 +20531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -20469,7 +20601,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -20493,27 +20625,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>42.67</v>
+        <v>41.9</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>43.61</v>
+        <v>42.42</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>44.53</v>
+        <v>42.91</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>09/10/2026 21:38:41</t>
+          <t>14/10/2026 18:28:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -20523,7 +20655,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PANGASIUS</t>
+          <t>TAMBAQUI</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -20537,27 +20669,27 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>9</v>
+        <v>11.5</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>9.5</v>
+        <v>11.7</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>09/10/2026 21:38:41</t>
+          <t>14/10/2026 18:28:17</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -20567,7 +20699,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>TAMBAQUI</t>
+          <t>TILÁPIA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -20581,113 +20713,25 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>11</v>
+        <v>11.87</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>11.5</v>
+        <v>12.14</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>12</v>
+        <v>12.38</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>09/10/2026 21:38:41</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>09/10/2026</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>TILÁPIA</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>11.71</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>12.08</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>12.39</v>
-      </c>
-      <c r="I5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>09/10/2026 21:38:41</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>09/10/2026</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>TRUTA</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>34.2</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>35.2</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>36.2</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>09/10/2026 21:38:41</t>
+          <t>14/10/2026 18:28:17</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J6"/>
+  <autoFilter ref="A1:J4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 16/10/2026 17:46
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$456</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$461</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J456"/>
+  <dimension ref="A1:J461"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -20519,8 +20519,228 @@
         </is>
       </c>
     </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F457" s="2" t="n">
+        <v>40.38</v>
+      </c>
+      <c r="G457" s="2" t="n">
+        <v>40.99</v>
+      </c>
+      <c r="H457" s="2" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="I457" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J457" t="inlineStr">
+        <is>
+          <t>16/10/2026 17:46:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F458" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="G458" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="H458" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="I458" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J458" t="inlineStr">
+        <is>
+          <t>16/10/2026 17:46:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F459" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="G459" s="2" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="H459" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="I459" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J459" t="inlineStr">
+        <is>
+          <t>16/10/2026 17:46:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F460" s="2" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="G460" s="2" t="n">
+        <v>12.23</v>
+      </c>
+      <c r="H460" s="2" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="I460" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J460" t="inlineStr">
+        <is>
+          <t>16/10/2026 17:46:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F461" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="G461" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="H461" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="I461" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J461" t="inlineStr">
+        <is>
+          <t>16/10/2026 17:46:56</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J456"/>
+  <autoFilter ref="A1:J461"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -20531,7 +20751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -20601,7 +20821,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -20625,27 +20845,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>41.9</v>
+        <v>40.38</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>42.42</v>
+        <v>40.99</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>42.91</v>
+        <v>41.6</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>14/10/2026 18:28:17</t>
+          <t>16/10/2026 17:46:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -20655,7 +20875,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>TAMBAQUI</t>
+          <t>PINTADO</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -20669,27 +20889,27 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>11.5</v>
+        <v>26</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>11.7</v>
+        <v>27</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>14/10/2026 18:28:17</t>
+          <t>16/10/2026 17:46:56</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -20699,39 +20919,127 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>16/10/2026 17:46:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>TILÁPIA</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>11.87</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>12.14</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>12.38</v>
-      </c>
-      <c r="I4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>14/10/2026 18:28:17</t>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>12.23</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>16/10/2026 17:46:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>16/10/2026 17:46:56</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J4"/>
+  <autoFilter ref="A1:J6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 19/10/2026 21:10
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$461</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$466</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J461"/>
+  <dimension ref="A1:J466"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -20739,8 +20739,228 @@
         </is>
       </c>
     </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F462" s="2" t="n">
+        <v>40.33</v>
+      </c>
+      <c r="G462" s="2" t="n">
+        <v>40.92</v>
+      </c>
+      <c r="H462" s="2" t="n">
+        <v>41.51</v>
+      </c>
+      <c r="I462" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J462" t="inlineStr">
+        <is>
+          <t>19/10/2026 21:10:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F463" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="G463" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="H463" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="I463" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J463" t="inlineStr">
+        <is>
+          <t>19/10/2026 21:10:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F464" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="G464" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="H464" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="I464" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J464" t="inlineStr">
+        <is>
+          <t>19/10/2026 21:10:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F465" s="2" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="G465" s="2" t="n">
+        <v>12.14</v>
+      </c>
+      <c r="H465" s="2" t="n">
+        <v>12.41</v>
+      </c>
+      <c r="I465" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J465" t="inlineStr">
+        <is>
+          <t>19/10/2026 21:10:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F466" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="G466" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="H466" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="I466" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J466" t="inlineStr">
+        <is>
+          <t>19/10/2026 21:10:30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J461"/>
+  <autoFilter ref="A1:J466"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -20821,7 +21041,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>16/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -20845,27 +21065,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>40.38</v>
+        <v>40.33</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>40.99</v>
+        <v>40.92</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>41.6</v>
+        <v>41.51</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>16/10/2026 17:46:56</t>
+          <t>19/10/2026 21:10:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>16/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -20902,14 +21122,14 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>16/10/2026 17:46:56</t>
+          <t>19/10/2026 21:10:30</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>16/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -20936,24 +21156,24 @@
         <v>12</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>12.5</v>
+        <v>13</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>16/10/2026 17:46:56</t>
+          <t>19/10/2026 21:10:30</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>16/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -20977,27 +21197,27 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>11.92</v>
+        <v>11.8</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>12.23</v>
+        <v>12.14</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>12.5</v>
+        <v>12.41</v>
       </c>
       <c r="I5" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>16/10/2026 17:46:56</t>
+          <t>19/10/2026 21:10:30</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>16/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -21021,20 +21241,20 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I6" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>16/10/2026 17:46:56</t>
+          <t>19/10/2026 21:10:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 21/10/2026 18:27
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$466</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$470</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J466"/>
+  <dimension ref="A1:J470"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -20959,8 +20959,184 @@
         </is>
       </c>
     </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F467" s="2" t="n">
+        <v>39.93</v>
+      </c>
+      <c r="G467" s="2" t="n">
+        <v>40.44</v>
+      </c>
+      <c r="H467" s="2" t="n">
+        <v>40.96</v>
+      </c>
+      <c r="I467" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J467" t="inlineStr">
+        <is>
+          <t>21/10/2026 18:27:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F468" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="G468" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="H468" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="I468" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J468" t="inlineStr">
+        <is>
+          <t>21/10/2026 18:27:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F469" s="2" t="n">
+        <v>11.72</v>
+      </c>
+      <c r="G469" s="2" t="n">
+        <v>12.08</v>
+      </c>
+      <c r="H469" s="2" t="n">
+        <v>12.36</v>
+      </c>
+      <c r="I469" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J469" t="inlineStr">
+        <is>
+          <t>21/10/2026 18:27:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F470" s="2" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="G470" s="2" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="H470" s="2" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="I470" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J470" t="inlineStr">
+        <is>
+          <t>21/10/2026 18:27:34</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J466"/>
+  <autoFilter ref="A1:J470"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -20971,7 +21147,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -21041,7 +21217,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -21065,27 +21241,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>40.33</v>
+        <v>39.93</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>40.92</v>
+        <v>40.44</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>41.51</v>
+        <v>40.96</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>19/10/2026 21:10:30</t>
+          <t>21/10/2026 18:27:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -21122,14 +21298,14 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>19/10/2026 21:10:30</t>
+          <t>21/10/2026 18:27:34</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -21139,7 +21315,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>TAMBAQUI</t>
+          <t>TILÁPIA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -21153,27 +21329,27 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>12</v>
+        <v>11.72</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>13</v>
+        <v>12.08</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>14</v>
+        <v>12.36</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>19/10/2026 21:10:30</t>
+          <t>21/10/2026 18:27:34</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -21183,7 +21359,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>TILÁPIA</t>
+          <t>TRUTA</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -21197,69 +21373,25 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>11.8</v>
+        <v>36.5</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>12.14</v>
+        <v>37.5</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>12.41</v>
+        <v>38.5</v>
       </c>
       <c r="I5" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>19/10/2026 21:10:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>19/10/2026</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>TRUTA</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>37</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>19/10/2026 21:10:30</t>
+          <t>21/10/2026 18:27:34</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J6"/>
+  <autoFilter ref="A1:J5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 23/10/2026 18:14
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$470</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$474</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J470"/>
+  <dimension ref="A1:J474"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -21135,8 +21135,184 @@
         </is>
       </c>
     </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F471" s="2" t="n">
+        <v>39.93</v>
+      </c>
+      <c r="G471" s="2" t="n">
+        <v>40.44</v>
+      </c>
+      <c r="H471" s="2" t="n">
+        <v>40.96</v>
+      </c>
+      <c r="I471" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J471" t="inlineStr">
+        <is>
+          <t>23/10/2026 18:14:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F472" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="G472" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="H472" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="I472" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J472" t="inlineStr">
+        <is>
+          <t>23/10/2026 18:14:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F473" s="2" t="n">
+        <v>11.72</v>
+      </c>
+      <c r="G473" s="2" t="n">
+        <v>12.08</v>
+      </c>
+      <c r="H473" s="2" t="n">
+        <v>12.36</v>
+      </c>
+      <c r="I473" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J473" t="inlineStr">
+        <is>
+          <t>23/10/2026 18:14:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F474" s="2" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="G474" s="2" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="H474" s="2" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="I474" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J474" t="inlineStr">
+        <is>
+          <t>23/10/2026 18:14:32</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J470"/>
+  <autoFilter ref="A1:J474"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -21217,7 +21393,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>23/10/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -21254,14 +21430,14 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>21/10/2026 18:27:34</t>
+          <t>23/10/2026 18:14:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>23/10/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -21298,14 +21474,14 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>21/10/2026 18:27:34</t>
+          <t>23/10/2026 18:14:32</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>23/10/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -21342,14 +21518,14 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>21/10/2026 18:27:34</t>
+          <t>23/10/2026 18:14:32</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>23/10/2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -21386,7 +21562,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>21/10/2026 18:27:34</t>
+          <t>23/10/2026 18:14:32</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 26/10/2026 21:18
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$474</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$480</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J474"/>
+  <dimension ref="A1:J480"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -21311,8 +21311,272 @@
         </is>
       </c>
     </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>26/10/2026</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F475" s="2" t="n">
+        <v>40.28</v>
+      </c>
+      <c r="G475" s="2" t="n">
+        <v>40.79</v>
+      </c>
+      <c r="H475" s="2" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="I475" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J475" t="inlineStr">
+        <is>
+          <t>26/10/2026 21:18:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>26/10/2026</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>PANGASIUS</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F476" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="G476" s="2" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H476" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I476" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J476" t="inlineStr">
+        <is>
+          <t>26/10/2026 21:18:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>26/10/2026</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F477" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="G477" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="H477" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="I477" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J477" t="inlineStr">
+        <is>
+          <t>26/10/2026 21:18:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>26/10/2026</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F478" s="2" t="n">
+        <v>11.15</v>
+      </c>
+      <c r="G478" s="2" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="H478" s="2" t="n">
+        <v>12.23</v>
+      </c>
+      <c r="I478" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J478" t="inlineStr">
+        <is>
+          <t>26/10/2026 21:18:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>26/10/2026</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F479" s="2" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="G479" s="2" t="n">
+        <v>12.17</v>
+      </c>
+      <c r="H479" s="2" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="I479" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J479" t="inlineStr">
+        <is>
+          <t>26/10/2026 21:18:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>26/10/2026</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>TRUTA</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F480" s="2" t="n">
+        <v>36.93</v>
+      </c>
+      <c r="G480" s="2" t="n">
+        <v>37.93</v>
+      </c>
+      <c r="H480" s="2" t="n">
+        <v>38.93</v>
+      </c>
+      <c r="I480" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J480" t="inlineStr">
+        <is>
+          <t>26/10/2026 21:18:12</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J474"/>
+  <autoFilter ref="A1:J480"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -21323,7 +21587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -21393,7 +21657,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>26/10/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -21417,27 +21681,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>39.93</v>
+        <v>40.28</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>40.44</v>
+        <v>40.79</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>40.96</v>
+        <v>41.3</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>23/10/2026 18:14:32</t>
+          <t>26/10/2026 21:18:12</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>26/10/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -21447,7 +21711,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PINTADO</t>
+          <t>PANGASIUS</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -21461,27 +21725,27 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>27</v>
+        <v>9.5</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>23/10/2026 18:14:32</t>
+          <t>26/10/2026 21:18:12</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>26/10/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -21491,7 +21755,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>TILÁPIA</t>
+          <t>PINTADO</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -21505,27 +21769,27 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>11.72</v>
+        <v>26</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>12.08</v>
+        <v>27</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>12.36</v>
+        <v>28</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>23/10/2026 18:14:32</t>
+          <t>26/10/2026 21:18:12</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>26/10/2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -21535,39 +21799,127 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>11.15</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>12.23</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>26/10/2026 21:18:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>26/10/2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>12.17</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>26/10/2026 21:18:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>26/10/2026</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>TRUTA</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>36.5</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>38.5</v>
-      </c>
-      <c r="I5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>23/10/2026 18:14:32</t>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>36.93</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>37.93</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>38.93</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>26/10/2026 21:18:12</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J5"/>
+  <autoFilter ref="A1:J7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 28/10/2026 21:41
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$480</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$482</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J480"/>
+  <dimension ref="A1:J482"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -21575,8 +21575,96 @@
         </is>
       </c>
     </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F481" s="2" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="G481" s="2" t="n">
+        <v>40.79</v>
+      </c>
+      <c r="H481" s="2" t="n">
+        <v>41.67</v>
+      </c>
+      <c r="I481" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J481" t="inlineStr">
+        <is>
+          <t>28/10/2026 21:41:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F482" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="G482" s="2" t="n">
+        <v>12.49</v>
+      </c>
+      <c r="H482" s="2" t="n">
+        <v>12.98</v>
+      </c>
+      <c r="I482" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J482" t="inlineStr">
+        <is>
+          <t>28/10/2026 21:41:39</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J480"/>
+  <autoFilter ref="A1:J482"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -21587,7 +21675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -21657,7 +21745,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>26/10/2026</t>
+          <t>28/10/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -21681,27 +21769,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>40.28</v>
+        <v>39.9</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>40.79</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>41.3</v>
+        <v>41.67</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>26/10/2026 21:18:12</t>
+          <t>28/10/2026 21:41:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>26/10/2026</t>
+          <t>28/10/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -21711,7 +21799,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PANGASIUS</t>
+          <t>TILÁPIA</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -21725,201 +21813,25 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>9.5</v>
+        <v>12.49</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>10</v>
+        <v>12.98</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>26/10/2026 21:18:12</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>26/10/2026</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>PINTADO</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="I4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>26/10/2026 21:18:12</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>26/10/2026</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>TAMBAQUI</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>11.15</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>11.7</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>12.23</v>
-      </c>
-      <c r="I5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>26/10/2026 21:18:12</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>26/10/2026</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>TILÁPIA</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>11.9</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>12.17</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>12.4</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>26/10/2026 21:18:12</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>26/10/2026</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>PESCADOS</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>TRUTA</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>36.93</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>37.93</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>38.93</v>
-      </c>
-      <c r="I7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>26/10/2026 21:18:12</t>
+          <t>28/10/2026 21:41:39</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J7"/>
+  <autoFilter ref="A1:J3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cotacoes CEAGESP - coleta de 30/10/2026 19:06
</commit_message>
<xml_diff>
--- a/dados/cotacoes_pescado.xlsx
+++ b/dados/cotacoes_pescado.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Ultimo boletim" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$482</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historico'!$A$1:$J$487</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ultimo boletim'!$A$1:$J$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J482"/>
+  <dimension ref="A1:J487"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -21663,8 +21663,228 @@
         </is>
       </c>
     </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>FILE DE TILAPIA</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F483" s="2" t="n">
+        <v>41.67</v>
+      </c>
+      <c r="G483" s="2" t="n">
+        <v>42.34</v>
+      </c>
+      <c r="H483" s="2" t="n">
+        <v>43.02</v>
+      </c>
+      <c r="I483" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J483" t="inlineStr">
+        <is>
+          <t>30/10/2026 19:06:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>PANGASIUS</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F484" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="G484" s="2" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H484" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="I484" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J484" t="inlineStr">
+        <is>
+          <t>30/10/2026 19:06:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F485" s="2" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="G485" s="2" t="n">
+        <v>23.98</v>
+      </c>
+      <c r="H485" s="2" t="n">
+        <v>24.54</v>
+      </c>
+      <c r="I485" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J485" t="inlineStr">
+        <is>
+          <t>30/10/2026 19:06:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F486" s="2" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="G486" s="2" t="n">
+        <v>11.79</v>
+      </c>
+      <c r="H486" s="2" t="n">
+        <v>12.35</v>
+      </c>
+      <c r="I486" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J486" t="inlineStr">
+        <is>
+          <t>30/10/2026 19:06:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>TILÁPIA</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F487" s="2" t="n">
+        <v>11.22</v>
+      </c>
+      <c r="G487" s="2" t="n">
+        <v>11.62</v>
+      </c>
+      <c r="H487" s="2" t="n">
+        <v>12.05</v>
+      </c>
+      <c r="I487" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J487" t="inlineStr">
+        <is>
+          <t>30/10/2026 19:06:34</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J482"/>
+  <autoFilter ref="A1:J487"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -21675,7 +21895,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -21745,7 +21965,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>28/10/2026</t>
+          <t>30/10/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -21769,27 +21989,27 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>39.9</v>
+        <v>41.67</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>40.79</v>
+        <v>42.34</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>41.67</v>
+        <v>43.02</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>28/10/2026 21:41:39</t>
+          <t>30/10/2026 19:06:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>28/10/2026</t>
+          <t>30/10/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -21799,39 +22019,171 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>PANGASIUS</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>30/10/2026 19:06:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>PINTADO</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>23.98</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>24.54</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>30/10/2026 19:06:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TAMBAQUI</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>11.79</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>12.35</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>30/10/2026 19:06:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PESCADOS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>TILÁPIA</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>12.49</v>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>12.98</v>
-      </c>
-      <c r="I3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>28/10/2026 21:41:39</t>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>11.22</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>11.62</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>12.05</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>30/10/2026 19:06:34</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J3"/>
+  <autoFilter ref="A1:J6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>